<commit_message>
G6.1: rebuild Home Safety spec on Foster City Village's programme; add Hassett partner
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hvHoqEQfyfe3Cs5LEBeem
</commit_message>
<xml_diff>
--- a/gaps/ThriveAtHome_Gap_Build_Tracker.xlsx
+++ b/gaps/ThriveAtHome_Gap_Build_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="236">
   <si>
     <t xml:space="preserve">ThriveAtHome Gap Build Tracker — G1 to G4 (40 phases)</t>
   </si>
@@ -445,10 +445,10 @@
     <t xml:space="preserve">G6.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Home Safety Program</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home safety checks (in person or virtual $49), report, fixes routed to volunteers/providers/partners, follow-up</t>
+    <t xml:space="preserve">Home Safety &amp; Earthquake Prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelled on Foster City Village: yearly programme, volunteers with 3–5 homes, training, inspection, itemised proposal (all/some/none), licensed contractor work, free/subsidised/member-pays costs, fridge magnet, Go-Bag, presentation series, grant report</t>
   </si>
   <si>
     <t xml:space="preserve">G6.2</t>
@@ -520,6 +520,18 @@
     <t xml:space="preserve">Confirmed? (Y/N)</t>
   </si>
   <si>
+    <t xml:space="preserve">Hassett Hardware — Handyman Program</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Mateo (Foster City)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Licensed contractor partner in Foster City Village's home safety programme</t>
+  </si>
+  <si>
     <t xml:space="preserve">HIP Housing — Home Sharing Program</t>
   </si>
   <si>
@@ -557,9 +569,6 @@
   </si>
   <si>
     <t xml:space="preserve">San Mateo; Marin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm</t>
   </si>
   <si>
     <t xml:space="preserve">Paid part-time community service training for low-income adults 55+</t>
@@ -2097,7 +2106,7 @@
       </c>
       <c r="G45" s="6"/>
     </row>
-    <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
         <v>135</v>
       </c>
@@ -2288,7 +2297,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -2328,12 +2337,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>165</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>166</v>
@@ -2347,12 +2356,12 @@
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
     </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>169</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>170</v>
@@ -2374,26 +2383,26 @@
         <v>139</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>178</v>
@@ -2412,48 +2421,48 @@
         <v>145</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>103</v>
+        <v>145</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>186</v>
@@ -2472,7 +2481,7 @@
         <v>188</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>189</v>
@@ -2488,20 +2497,39 @@
         <v>145</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
     </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F12" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F13" type="list">
       <formula1>"Y,N"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2531,84 +2559,84 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2636,79 +2664,79 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>